<commit_message>
paper run 2026-10-12 10:22
</commit_message>
<xml_diff>
--- a/reports/2026-10-12.xlsx
+++ b/reports/2026-10-12.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,135 @@
       </c>
       <c r="K3" t="n">
         <v>22.05</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-12T04:48:50.366085+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.5344</v>
+      </c>
+      <c r="F4" t="n">
+        <v>42.97</v>
+      </c>
+      <c r="G4" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.761</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.00102</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>-42.97</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-12T05:11:22.385825+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F5" t="n">
+        <v>20.54</v>
+      </c>
+      <c r="G5" t="n">
+        <v>40.27</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.762</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.00115</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>19.73</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-12T09:38:54.952823+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F6" t="n">
+        <v>16.87</v>
+      </c>
+      <c r="G6" t="n">
+        <v>28.11</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.771</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.00121</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>-16.87</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,7 +722,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -603,7 +732,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -613,7 +742,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -623,7 +752,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="6">
@@ -633,7 +762,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>17.73</v>
+        <v>-22.38</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +772,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>22.05</v>
+        <v>41.78</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +782,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-4.32</v>
+        <v>-64.16</v>
       </c>
     </row>
     <row r="9">
@@ -663,7 +792,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5.1</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="10">
@@ -673,7 +802,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3161.319999999999</v>
+        <v>3121.209999999999</v>
       </c>
     </row>
     <row r="12">
@@ -724,256 +853,272 @@
         </is>
       </c>
       <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="n">
         <v>2</v>
       </c>
-      <c r="C15" t="n">
-        <v>1</v>
-      </c>
       <c r="D15" t="n">
-        <v>-6.37</v>
+        <v>143.43</v>
       </c>
       <c r="E15" t="n">
-        <v>17.73</v>
+        <v>37.46</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-286.42</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-59.84</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" t="n">
-        <v>-157.18</v>
-      </c>
-      <c r="E17" t="n">
-        <v>-4.32</v>
+          <t>По активам</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>150.81</v>
+        <v>-155.3</v>
       </c>
       <c r="E18" t="n">
-        <v>22.05</v>
+        <v>-27.56</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>12.31</v>
+      </c>
+      <c r="E19" t="n">
+        <v>5.18</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>2</v>
-      </c>
-      <c r="C20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" t="n">
-        <v>-6.37</v>
-      </c>
-      <c r="E20" t="n">
-        <v>17.73</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>-4.49</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-5.51</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>-6.37</v>
+        <v>-138.5</v>
       </c>
       <c r="E22" t="n">
-        <v>17.73</v>
+        <v>-16.87</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>5</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-142.99</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-22.38</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>1</v>
-      </c>
-      <c r="C27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" t="n">
-        <v>-4.32</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" t="n">
-        <v>22.05</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>-27.56</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>2</v>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>5.18</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>По окнам</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>2</v>
-      </c>
-      <c r="C31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" t="n">
-        <v>17.73</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>3</v>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="n">
+        <v>37.46</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>5m</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>2</v>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>17.73</v>
+        <v>-59.84</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>По цене входа</t>
+          <t>По часам</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -995,7 +1140,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1008,96 +1153,230 @@
         <v>17.73</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>-42.97</v>
+      </c>
+    </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>19.73</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>09</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>22.05</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>0.15–0.20%</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="n">
-        <v>0</v>
-      </c>
-      <c r="D41" t="n">
-        <v>-4.32</v>
+        <v>-16.87</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>4</v>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" t="n">
+        <v>-5.51</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="n">
+        <v>-16.87</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>3</v>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="n">
+        <v>-1.19</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" t="n">
+        <v>-16.87</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" t="n">
+        <v>-4.32</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="B52" t="n">
         <v>2</v>
       </c>
-      <c r="C44" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" t="n">
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
         <v>17.73</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>3</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>-40.11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-10-12 20:17
</commit_message>
<xml_diff>
--- a/reports/2026-10-12.xlsx
+++ b/reports/2026-10-12.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -853,13 +853,13 @@
         </is>
       </c>
       <c r="B15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="n">
         <v>3</v>
       </c>
-      <c r="C15" t="n">
-        <v>2</v>
-      </c>
       <c r="D15" t="n">
-        <v>143.43</v>
+        <v>266.05</v>
       </c>
       <c r="E15" t="n">
         <v>37.46</v>
@@ -872,13 +872,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>-286.42</v>
+        <v>-148.03</v>
       </c>
       <c r="E16" t="n">
         <v>-59.84</v>
@@ -898,13 +898,13 @@
         </is>
       </c>
       <c r="B18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" t="n">
         <v>3</v>
       </c>
-      <c r="C18" t="n">
-        <v>1</v>
-      </c>
       <c r="D18" t="n">
-        <v>-155.3</v>
+        <v>105.71</v>
       </c>
       <c r="E18" t="n">
         <v>-27.56</v>
@@ -943,13 +943,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>-4.49</v>
+        <v>133.9</v>
       </c>
       <c r="E21" t="n">
         <v>-5.51</v>
@@ -962,13 +962,13 @@
         </is>
       </c>
       <c r="B22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="n">
         <v>1</v>
       </c>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
       <c r="D22" t="n">
-        <v>-138.5</v>
+        <v>-15.88</v>
       </c>
       <c r="E22" t="n">
         <v>-16.87</v>
@@ -984,335 +984,338 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NO_LIQUIDITY</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C24" t="n">
         <v>2</v>
       </c>
       <c r="D24" t="n">
+        <v>261.01</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>5</v>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" t="n">
         <v>-142.99</v>
       </c>
-      <c r="E24" t="n">
+      <c r="E25" t="n">
         <v>-22.38</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>3</v>
-      </c>
-      <c r="C29" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" t="n">
-        <v>-27.56</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C30" t="n">
         <v>1</v>
       </c>
       <c r="D30" t="n">
+        <v>-27.56</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
         <v>5.18</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>3</v>
-      </c>
-      <c r="C33" t="n">
-        <v>2</v>
-      </c>
-      <c r="D33" t="n">
-        <v>37.46</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" t="n">
+        <v>37.46</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>5m</t>
         </is>
       </c>
-      <c r="B34" t="n">
+      <c r="B35" t="n">
         <v>2</v>
       </c>
-      <c r="C34" t="n">
+      <c r="C35" t="n">
         <v>0</v>
       </c>
-      <c r="D34" t="n">
+      <c r="D35" t="n">
         <v>-59.84</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>2</v>
-      </c>
-      <c r="C37" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" t="n">
-        <v>17.73</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" t="n">
         <v>1</v>
       </c>
-      <c r="C38" t="n">
-        <v>0</v>
-      </c>
       <c r="D38" t="n">
-        <v>-42.97</v>
+        <v>17.73</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>19.73</v>
+        <v>-42.97</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>1</v>
       </c>
       <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>19.73</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
         <v>0</v>
       </c>
-      <c r="D40" t="n">
+      <c r="D41" t="n">
         <v>-16.87</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>4</v>
-      </c>
-      <c r="C43" t="n">
-        <v>2</v>
-      </c>
-      <c r="D43" t="n">
-        <v>-5.51</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>4</v>
+      </c>
+      <c r="C44" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" t="n">
+        <v>-5.51</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>0.55–0.60</t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="B45" t="n">
         <v>1</v>
       </c>
-      <c r="C44" t="n">
+      <c r="C45" t="n">
         <v>0</v>
       </c>
-      <c r="D44" t="n">
+      <c r="D45" t="n">
         <v>-16.87</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>3</v>
-      </c>
-      <c r="C47" t="n">
-        <v>2</v>
-      </c>
-      <c r="D47" t="n">
-        <v>-1.19</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D48" t="n">
-        <v>-16.87</v>
+        <v>-1.19</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
+          <t>0.12–0.15%</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1322,60 +1325,76 @@
         <v>0</v>
       </c>
       <c r="D49" t="n">
+        <v>-16.87</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" t="n">
         <v>-4.32</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>2</v>
-      </c>
-      <c r="C52" t="n">
-        <v>1</v>
-      </c>
-      <c r="D52" t="n">
-        <v>17.73</v>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C53" t="n">
         <v>1</v>
       </c>
       <c r="D53" t="n">
+        <v>17.73</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="n">
         <v>-40.11</v>
       </c>
     </row>

</xml_diff>